<commit_message>
Printable pack and Money Reset Kit bundle
- product_print.py: six pen-and-paper pages (paycheck split, subscription audit, sinking funds, debt list,
  net worth, how-to) in US Letter and A4 PDF; a check proves nothing is drawn in the printer-unsafe margins.
- Bundle: both planners + printables with read-me and licence, and a listing with test prices marked as
  assumptions. `python -m faceless products` now builds, verifies and ships all four.
- empire: P3 and P4 built.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016paNQMdrshJA9eY2StVQcF
</commit_message>
<xml_diff>
--- a/channel/products/rat-race-escape-planner/Rat-Race-Escape-Planner.xlsx
+++ b/channel/products/rat-race-escape-planner/Rat-Race-Escape-Planner.xlsx
@@ -1427,11 +1427,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="93365701"/>
-        <c:axId val="46833287"/>
+        <c:axId val="30425755"/>
+        <c:axId val="44964645"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="93365701"/>
+        <c:axId val="30425755"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1463,7 +1463,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46833287"/>
+        <c:crossAx val="44964645"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1471,7 +1471,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46833287"/>
+        <c:axId val="44964645"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1513,7 +1513,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93365701"/>
+        <c:crossAx val="30425755"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>